<commit_message>
kengo 5 13 12:09
</commit_message>
<xml_diff>
--- a/作業票.xlsx
+++ b/作業票.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\coop2\Project-Chi2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Sasaki Kengo\Project-Chi2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1DD8D650-C74E-4A75-AE8E-E75212413C83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B78A639-F959-4C66-B926-B67CA37A4E20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13875" xr2:uid="{41B48087-E4EE-4E9E-AF83-941FF13AEAD0}"/>
   </bookViews>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="25">
   <si>
     <t>タスク</t>
     <phoneticPr fontId="1"/>
@@ -238,6 +238,16 @@
     </rPh>
     <rPh sb="19" eb="22">
       <t>ヨウソウダン</t>
+    </rPh>
+    <phoneticPr fontId="1"/>
+  </si>
+  <si>
+    <t>敵の攻撃</t>
+    <rPh sb="0" eb="1">
+      <t>テキ</t>
+    </rPh>
+    <rPh sb="2" eb="4">
+      <t>コウゲキ</t>
     </rPh>
     <phoneticPr fontId="1"/>
   </si>
@@ -1008,10 +1018,14 @@
       <c r="B7" s="8">
         <v>5</v>
       </c>
-      <c r="C7" s="4"/>
-      <c r="D7" s="3"/>
+      <c r="C7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>16</v>
+      </c>
       <c r="E7" s="1" t="s">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="F7" s="10"/>
     </row>

</xml_diff>